<commit_message>
Weekly refresh (2026-10-31) follow-up — RGT re-verified (shallow-check reset missed from first pass)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trust_urls.xlsx
+++ b/trust_urls.xlsx
@@ -7393,7 +7393,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7403,7 +7403,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Re-verified 2026-10-10 by local curl: landing links the 2026 year page, which lists event pages for 11 Mar, 10 Jun, 9 Sep and 9 Dec 2026.</t>
+          <t>Re-verified 2026-10-31 by local browser-UA curl (200, 82KB; the shallow scanner saw a transient connection reset): landing links the year pages (deep validator: 6 year archives); 2026 dates incl. 4 September 2026 shown.</t>
         </is>
       </c>
       <c r="P92" t="inlineStr"/>

</xml_diff>